<commit_message>
feat(question-loading): topic-based prompt v3, concept column, topic-block checks
The generator prompt now asks only for the level, breaks the source into
teacher-language topics with concepts, and writes blocks of 50 different
questions per topic (15 easy / 20 medium / 15 hard) in batches of 100 rows, with
explanations that teach. Template gains a concept column (20 columns) and topic
is required everywhere. The checker reports each topic's block size, difficulty
spread, concept coverage and name variants. Tracker gains track T (topic
registry, even-spread assignments, study mode, understanding measure).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/question-loading/QuizBox_Question_Load_Template.xlsx
+++ b/docs/question-loading/QuizBox_Question_Load_Template.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -442,18 +442,19 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="46" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,60 +495,65 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>cognitive_level</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>answer_type</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>question_text</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>option_a</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>option_b</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>option_c</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>option_d</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>correct_answer</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>explanation</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>source_reference</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>source_quote</t>
         </is>
@@ -558,16 +564,16 @@
     <dataValidation sqref="A2:A2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
       <formula1>"PRIMARY,JHS,SHS,SPONSOR"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
+    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
       <formula1>"easy,medium,hard"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
+    <dataValidation sqref="J2:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
       <formula1>"Remember,Understand,Apply,Analyse,Evaluate"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
+    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
       <formula1>"SINGLE_CHOICE,TRUE_FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
+    <dataValidation sqref="Q2:Q2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not allowed" error="Pick a value from the list." type="list">
       <formula1>"A,B,C,D"</formula1>
     </dataValidation>
   </dataValidations>
@@ -581,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -664,7 +670,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>e.g. Science, Mathematics, Computing</t>
+          <t>e.g. Science, Social Studies</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -674,7 +680,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Use the subject name exactly as listed in the loader's subject picker.</t>
+          <t>Subject name as it appears in the curriculum.</t>
         </is>
       </c>
     </row>
@@ -740,7 +746,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Learning-indicator code exactly as printed in the curriculum. This links the question to the curriculum.</t>
+          <t>Learning-indicator code exactly as printed in the curriculum. The topic belongs to this indicator.</t>
         </is>
       </c>
     </row>
@@ -752,51 +758,51 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teacher-language name</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Sponsor: required. Curriculum: optional</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>The topic or section of the source document that this question tests.</t>
+          <t>The topic a teacher would teach in one to three lessons (for example Components of maps). Every question in a topic uses exactly the same wording. A topic has a block of 50 questions.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>difficulty</t>
+          <t>concept</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>easy, medium or hard</t>
+          <t>short concept name</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Only these three words, lower case.</t>
+          <t>The one concept inside the topic that this question builds (3 to 8 concepts per topic, each with at least 3 questions). Used to show how much of the topic a learner understands.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>cognitive_level</t>
+          <t>difficulty</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Remember, Understand, Apply, Analyse, Evaluate</t>
+          <t>easy, medium or hard</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -806,19 +812,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Use one of the five words.</t>
+          <t>Only these three words, lower case. Per topic of 50: 15 easy, 20 medium, 15 hard.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>answer_type</t>
+          <t>cognitive_level</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SINGLE_CHOICE or TRUE_FALSE</t>
+          <t>Remember, Understand, Apply, Analyse, Evaluate</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -828,19 +834,19 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>TRUE_FALSE: option_a must be True and option_b must be False; leave C and D blank.</t>
+          <t>Use one of the five words.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>question_text</t>
+          <t>answer_type</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>plain text</t>
+          <t>SINGLE_CHOICE or TRUE_FALSE</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -850,14 +856,14 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>One clear question. No HTML, no &lt; or &gt; characters, no line breaks. Never write 'the answer is' or 'correct answer' in it.</t>
+          <t>TRUE_FALSE: option_a must be True and option_b must be False; leave C and D blank.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>option_a</t>
+          <t>question_text</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -872,14 +878,14 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>First option.</t>
+          <t>One clear question that stands on its own. No HTML, no &lt; or &gt; characters, no line breaks. Never write 'the answer is' or 'correct answer'.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>option_b</t>
+          <t>option_a</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -894,14 +900,14 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Second option.</t>
+          <t>First option.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>option_c</t>
+          <t>option_b</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -911,19 +917,19 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Required for SINGLE_CHOICE</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Third option. Blank for TRUE_FALSE.</t>
+          <t>Second option.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>option_d</t>
+          <t>option_c</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -938,41 +944,41 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Fourth option. Blank for TRUE_FALSE.</t>
+          <t>Third option. Blank for TRUE_FALSE.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>correct_answer</t>
+          <t>option_d</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>A, B, C or D</t>
+          <t>plain text</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required for SINGLE_CHOICE</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>The letter of the one correct option. For TRUE_FALSE use A (True) or B (False).</t>
+          <t>Fourth option. Blank for TRUE_FALSE.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>explanation</t>
+          <t>correct_answer</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>plain text</t>
+          <t>A, B, C or D</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -982,19 +988,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Why the correct answer is right and what makes the main wrong option wrong. Specific to this question.</t>
+          <t>The letter of the one correct option. For TRUE_FALSE use A (True) or B (False).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>source_reference</t>
+          <t>explanation</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>e.g. NaCCA Science B7 p.34, Strand 4</t>
+          <t>plain text, 20-60 words</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1004,27 +1010,49 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Where in the supplied document the question comes from (page, chapter or section).</t>
+          <t>Teaches the idea in plain words: why the answer is right and what the most tempting wrong option gets wrong. A learner who missed the lesson should understand from reading it.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>source_reference</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>e.g. NaCCA Social Studies B7 p.24</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Where in the supplied document the question comes from (page, chapter or section).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>source_quote</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Sponsor: required. Curriculum: recommended</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>A short phrase copied word for word from the supplied document that supports the answer.</t>
         </is>
@@ -1041,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1054,15 +1082,16 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="50" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1103,60 +1132,65 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>cognitive_level</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>answer_type</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>question_text</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>option_a</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>option_b</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>option_c</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>option_d</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>correct_answer</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>explanation</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>source_reference</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>source_quote</t>
         </is>
@@ -1175,87 +1209,92 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Forces and Energy</t>
+          <t>Strand 1: Environmental Issues</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Conversion and Conservation of Energy</t>
+          <t>Sub-Strand 2: Mapping Skills</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>B7.4.3.1.2</t>
+          <t>B7.1.2.1.1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>energy conversion</t>
+          <t>Components of maps</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>North arrow</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>Remember</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>SINGLE_CHOICE</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>A torch converts the chemical energy stored in its battery mainly into which two forms of energy?</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Light and heat</t>
+          <t>Which part of a map shows the direction of North?</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sound and light</t>
+          <t>The map key</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Kinetic and sound</t>
+          <t>The north arrow</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Chemical and heat</t>
+          <t>The scale bar</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>The title</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>A battery stores chemical energy. In the torch circuit it is converted into light from the bulb and heat from the filament. Sound and kinetic energy are not produced in a working torch.</t>
+          <t>B</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>NaCCA Science B7, Strand 4, Sub-strand 3</t>
+          <t>The north arrow points to North so you can tell which way the map is turned. The key explains symbols and the scale bar measures distance, so neither shows direction.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>conversion of energy into useable forms</t>
+          <t>NaCCA Social Studies B7 p.26</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Identify components of maps, including North arrow, scale, map key</t>
         </is>
       </c>
     </row>
@@ -1267,62 +1306,75 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chapter 2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Crossings</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Road safety: zebra crossings</t>
+          <t>Zebra crossings</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>Right of way</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Remember</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>TRUE_FALSE</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Drivers must stop for pedestrians who are on a zebra crossing.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>The sponsor's guide says drivers must give way to pedestrians on a marked zebra crossing.</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>The guide says drivers must give way to pedestrians on a marked zebra crossing, so the statement is true.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>Road Safety Guide, page 12</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>drivers must give way to pedestrians on a zebra crossing</t>
         </is>
@@ -1341,13 +1393,6 @@
   </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">

</xml_diff>